<commit_message>
feat(sow): bobot sub-task dihitung dari standard_hours + fitur 'Tambah dari Standar'
- migration 20260806: standard_hours di sow_sub_operation + sow_sub_operation_standard, weight jadi turunan (share jam), trigger autoseed salin jam
- fix 42P18: recompute pakai 2 param terpisah (progress integer vs actual_progress numeric)
- cap: SUM(jam sub-task) <= sow.planhours (400 bila lebih), skip bila planhours 0
- POST /sow/operations/:idsow/subtasks/batch: create massal atomik + dedupe judul + cap sekali (sow_management W)
- GET /sow/subtask-standards: filter operation_text; fix NORM regex (backslash ganda) — normalisasi spasi-ganda selama ini tak jalan
- FE: form Jam Standar (0 = tak dihitung), bobot persen read-only, tombol Dari Standar + modal dari master (part_number+operation_text)
- fix StrictMode: mountedRef di ProgressUpdatePage & OrderListPage (skeleton abadi di npm run dev)
</commit_message>
<xml_diff>
--- a/samples/excel/sub_task_upload_template.xlsx
+++ b/samples/excel/sub_task_upload_template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sub_task" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PETUNJUK" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="sub_task" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="PETUNJUK" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -497,7 +497,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>weight</t>
+          <t>standard_hours</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -728,12 +728,12 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>weight</t>
+          <t>standard_hours</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Opsional (default 1). Bobot roll-up: progres operasi = SUM(progress*weight)/SUM(weight) atas sub-task aktif. Angka &gt; 0.</t>
+          <t>Opsional (default 1). Jam standar sub-task. Bobot dihitung otomatis = jam / total jam sub-task aktif; roll-up = SUM(progress x jam) / SUM(jam). 0 = sub-task tak dihitung. Total jam tidak boleh melebihi jam operasi.</t>
         </is>
       </c>
     </row>

</xml_diff>